<commit_message>
updates to sim and hi code
</commit_message>
<xml_diff>
--- a/contaminated_lognormal_final_summary.xlsx
+++ b/contaminated_lognormal_final_summary.xlsx
@@ -1,129 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user-pc\OneDrive\Documents\RP\Contaminated-log-normal-model-of-household-income-\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F98806-06EC-4424-95BE-653C422BF7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
     <sheet name="diagnostics" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>lambda_true</t>
-  </si>
-  <si>
-    <t>epsilon_true</t>
-  </si>
-  <si>
-    <t>m_mean</t>
-  </si>
-  <si>
-    <t>m_bias</t>
-  </si>
-  <si>
-    <t>m_mse</t>
-  </si>
-  <si>
-    <t>sigma_mean</t>
-  </si>
-  <si>
-    <t>sigma_bias</t>
-  </si>
-  <si>
-    <t>sigma_mse</t>
-  </si>
-  <si>
-    <t>lambda_mean</t>
-  </si>
-  <si>
-    <t>lambda_bias</t>
-  </si>
-  <si>
-    <t>lambda_mse</t>
-  </si>
-  <si>
-    <t>epsilon_mean</t>
-  </si>
-  <si>
-    <t>epsilon_bias</t>
-  </si>
-  <si>
-    <t>epsilon_mse</t>
-  </si>
-  <si>
-    <t>conv_rate_reg</t>
-  </si>
-  <si>
-    <t>conv_rate_mode</t>
-  </si>
-  <si>
-    <t>aic_win_single</t>
-  </si>
-  <si>
-    <t>aic_win_mix_reg</t>
-  </si>
-  <si>
-    <t>aic_win_mix_mode</t>
-  </si>
-  <si>
-    <t>bic_win_single</t>
-  </si>
-  <si>
-    <t>bic_win_mix_reg</t>
-  </si>
-  <si>
-    <t>bic_win_mix_mode</t>
-  </si>
-  <si>
-    <t>n_valid_gap</t>
-  </si>
-  <si>
-    <t>mean_logLik_gap</t>
-  </si>
-  <si>
-    <t>min_logLik_gap</t>
-  </si>
-  <si>
-    <t>max_logLik_gap</t>
-  </si>
-  <si>
-    <t>mean_abs_logLik_gap</t>
-  </si>
-  <si>
-    <t>prop_gap_gt_small</t>
-  </si>
-  <si>
-    <t>prop_gap_gt_large</t>
-  </si>
-  <si>
-    <t>n_reg_better_reps</t>
-  </si>
-  <si>
-    <t>n_mode_better_reps</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,21 +64,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -223,7 +108,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -257,7 +142,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -292,10 +176,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -468,106 +351,128 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.5703125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_true</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon_true</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>m_mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>m_bias</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>m_mse</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sigma_mean</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>sigma_bias</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sigma_mse</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_mean</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_bias</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_mse</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon_mean</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon_bias</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon_mse</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>conv_rate_reg</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>conv_rate_mode</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>aic_win_single</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>aic_win_mix_reg</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>aic_win_mix_mode</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>bic_win_single</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>bic_win_mix_reg</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>bic_win_mix_mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2">
         <v>100</v>
       </c>
@@ -578,40 +483,40 @@
         <v>0.6</v>
       </c>
       <c r="D2">
-        <v>2.0184000000000002</v>
+        <v>2.0243</v>
       </c>
       <c r="E2">
-        <v>1.84E-2</v>
+        <v>0.0243</v>
       </c>
       <c r="F2">
-        <v>2.1000000000000001E-2</v>
+        <v>0.0216</v>
       </c>
       <c r="G2">
-        <v>0.50409999999999999</v>
+        <v>0.2647</v>
       </c>
       <c r="H2">
-        <v>4.1000000000000003E-3</v>
+        <v>0.0147</v>
       </c>
       <c r="I2">
-        <v>6.7999999999999996E-3</v>
+        <v>0.007</v>
       </c>
       <c r="J2">
-        <v>2.3599000000000001</v>
+        <v>2.2856</v>
       </c>
       <c r="K2">
-        <v>0.3599</v>
+        <v>0.2856</v>
       </c>
       <c r="L2">
-        <v>1.4926999999999999</v>
+        <v>1.2959</v>
       </c>
       <c r="M2">
-        <v>0.72399999999999998</v>
+        <v>0.7363</v>
       </c>
       <c r="N2">
-        <v>0.124</v>
+        <v>0.1363</v>
       </c>
       <c r="O2">
-        <v>5.8099999999999999E-2</v>
+        <v>0.0604</v>
       </c>
       <c r="P2">
         <v>1</v>
@@ -620,25 +525,25 @@
         <v>1</v>
       </c>
       <c r="R2">
-        <v>0.81599999999999995</v>
+        <v>0.82</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>0.082</v>
       </c>
       <c r="U2">
-        <v>0.96399999999999997</v>
+        <v>0.968</v>
       </c>
       <c r="V2">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="W2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3">
         <v>100</v>
       </c>
@@ -649,40 +554,40 @@
         <v>0.9</v>
       </c>
       <c r="D3">
-        <v>2.0211000000000001</v>
+        <v>2.0171</v>
       </c>
       <c r="E3">
-        <v>2.1100000000000001E-2</v>
+        <v>0.0171</v>
       </c>
       <c r="F3">
-        <v>1.7299999999999999E-2</v>
+        <v>0.0188</v>
       </c>
       <c r="G3">
-        <v>0.47070000000000001</v>
+        <v>0.2257</v>
       </c>
       <c r="H3">
-        <v>-2.93E-2</v>
+        <v>-0.0243</v>
       </c>
       <c r="I3">
-        <v>4.8999999999999998E-3</v>
+        <v>0.0042</v>
       </c>
       <c r="J3">
-        <v>2.0708000000000002</v>
+        <v>2.1227</v>
       </c>
       <c r="K3">
-        <v>7.0800000000000002E-2</v>
+        <v>0.1227</v>
       </c>
       <c r="L3">
-        <v>1.5526</v>
+        <v>2.6798</v>
       </c>
       <c r="M3">
-        <v>0.79720000000000002</v>
+        <v>0.7974</v>
       </c>
       <c r="N3">
-        <v>-0.1028</v>
+        <v>-0.1026</v>
       </c>
       <c r="O3">
-        <v>5.1499999999999997E-2</v>
+        <v>0.0518</v>
       </c>
       <c r="P3">
         <v>1</v>
@@ -691,25 +596,25 @@
         <v>1</v>
       </c>
       <c r="R3">
-        <v>0.872</v>
+        <v>0.89</v>
       </c>
       <c r="S3">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T3">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="U3">
-        <v>0.97399999999999998</v>
+        <v>0.982</v>
       </c>
       <c r="V3">
-        <v>0</v>
+        <v>0.014</v>
       </c>
       <c r="W3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.004</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4">
         <v>100</v>
       </c>
@@ -720,40 +625,40 @@
         <v>0.6</v>
       </c>
       <c r="D4">
-        <v>2.0043000000000002</v>
+        <v>2.0152</v>
       </c>
       <c r="E4">
-        <v>4.3E-3</v>
+        <v>0.0152</v>
       </c>
       <c r="F4">
-        <v>3.3799999999999997E-2</v>
+        <v>0.0311</v>
       </c>
       <c r="G4">
-        <v>0.49740000000000001</v>
+        <v>0.2568</v>
       </c>
       <c r="H4">
-        <v>-2.5999999999999999E-3</v>
+        <v>0.0068</v>
       </c>
       <c r="I4">
-        <v>7.1000000000000004E-3</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="J4">
-        <v>5.4942000000000002</v>
+        <v>5.4883</v>
       </c>
       <c r="K4">
-        <v>0.49419999999999997</v>
+        <v>0.4883</v>
       </c>
       <c r="L4">
-        <v>3.2581000000000002</v>
+        <v>3.0426</v>
       </c>
       <c r="M4">
-        <v>0.60799999999999998</v>
+        <v>0.6179</v>
       </c>
       <c r="N4">
-        <v>8.0000000000000002E-3</v>
+        <v>0.0179</v>
       </c>
       <c r="O4">
-        <v>1.0500000000000001E-2</v>
+        <v>0.0107</v>
       </c>
       <c r="P4">
         <v>1</v>
@@ -762,25 +667,25 @@
         <v>1</v>
       </c>
       <c r="R4">
-        <v>2.8000000000000001E-2</v>
+        <v>0.022</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>0.462</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>0.516</v>
       </c>
       <c r="U4">
-        <v>0.13400000000000001</v>
+        <v>0.132</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>0.428</v>
       </c>
       <c r="W4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5">
         <v>100</v>
       </c>
@@ -791,40 +696,40 @@
         <v>0.9</v>
       </c>
       <c r="D5">
-        <v>2.0049999999999999</v>
+        <v>2.0047</v>
       </c>
       <c r="E5">
-        <v>5.0000000000000001E-3</v>
+        <v>0.0047</v>
       </c>
       <c r="F5">
-        <v>1.84E-2</v>
+        <v>0.0163</v>
       </c>
       <c r="G5">
-        <v>0.47849999999999998</v>
+        <v>0.2345</v>
       </c>
       <c r="H5">
-        <v>-2.1499999999999998E-2</v>
+        <v>-0.0155</v>
       </c>
       <c r="I5">
-        <v>4.0000000000000001E-3</v>
+        <v>0.0032</v>
       </c>
       <c r="J5">
-        <v>5.3390000000000004</v>
+        <v>5.3048</v>
       </c>
       <c r="K5">
-        <v>0.33900000000000002</v>
+        <v>0.3048</v>
       </c>
       <c r="L5">
-        <v>3.7178</v>
+        <v>4.0297</v>
       </c>
       <c r="M5">
-        <v>0.85089999999999999</v>
+        <v>0.8515</v>
       </c>
       <c r="N5">
-        <v>-4.9099999999999998E-2</v>
+        <v>-0.0485</v>
       </c>
       <c r="O5">
-        <v>1.6E-2</v>
+        <v>0.0164</v>
       </c>
       <c r="P5">
         <v>1</v>
@@ -833,25 +738,25 @@
         <v>1</v>
       </c>
       <c r="R5">
-        <v>0.09</v>
+        <v>0.102</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="T5">
-        <v>0</v>
+        <v>0.428</v>
       </c>
       <c r="U5">
-        <v>0.22600000000000001</v>
+        <v>0.26</v>
       </c>
       <c r="V5">
-        <v>0</v>
+        <v>0.382</v>
       </c>
       <c r="W5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.358</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6">
         <v>1000</v>
       </c>
@@ -862,40 +767,40 @@
         <v>0.6</v>
       </c>
       <c r="D6">
-        <v>2.0013999999999998</v>
+        <v>1.9996</v>
       </c>
       <c r="E6">
-        <v>1.4E-3</v>
+        <v>-0.0004</v>
       </c>
       <c r="F6">
-        <v>2E-3</v>
+        <v>0.0022</v>
       </c>
       <c r="G6">
-        <v>0.50449999999999995</v>
+        <v>0.2556</v>
       </c>
       <c r="H6">
-        <v>4.4999999999999997E-3</v>
+        <v>0.0056</v>
       </c>
       <c r="I6">
-        <v>1.5E-3</v>
+        <v>0.0016</v>
       </c>
       <c r="J6">
-        <v>2.1208999999999998</v>
+        <v>2.1062</v>
       </c>
       <c r="K6">
-        <v>0.12089999999999999</v>
+        <v>0.1062</v>
       </c>
       <c r="L6">
-        <v>0.1492</v>
+        <v>0.1129</v>
       </c>
       <c r="M6">
-        <v>0.63590000000000002</v>
+        <v>0.6355</v>
       </c>
       <c r="N6">
-        <v>3.5900000000000001E-2</v>
+        <v>0.0355</v>
       </c>
       <c r="O6">
-        <v>2.47E-2</v>
+        <v>0.0234</v>
       </c>
       <c r="P6">
         <v>1</v>
@@ -904,25 +809,25 @@
         <v>1</v>
       </c>
       <c r="R6">
-        <v>0.152</v>
+        <v>0.154</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>0.424</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <v>0.422</v>
       </c>
       <c r="U6">
-        <v>0.69</v>
+        <v>0.696</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="W6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.154</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -933,40 +838,40 @@
         <v>0.9</v>
       </c>
       <c r="D7">
-        <v>2.0011000000000001</v>
+        <v>1.9981</v>
       </c>
       <c r="E7">
-        <v>1.1000000000000001E-3</v>
+        <v>-0.0019</v>
       </c>
       <c r="F7">
-        <v>1.6000000000000001E-3</v>
+        <v>0.0017</v>
       </c>
       <c r="G7">
-        <v>0.48570000000000002</v>
+        <v>0.2378</v>
       </c>
       <c r="H7">
-        <v>-1.43E-2</v>
+        <v>-0.0122</v>
       </c>
       <c r="I7">
-        <v>1.1999999999999999E-3</v>
+        <v>0.0011</v>
       </c>
       <c r="J7">
-        <v>2.1941999999999999</v>
+        <v>2.1423</v>
       </c>
       <c r="K7">
-        <v>0.19420000000000001</v>
+        <v>0.1423</v>
       </c>
       <c r="L7">
-        <v>0.69810000000000005</v>
+        <v>0.5876</v>
       </c>
       <c r="M7">
-        <v>0.79820000000000002</v>
+        <v>0.7875</v>
       </c>
       <c r="N7">
-        <v>-0.1018</v>
+        <v>-0.1125</v>
       </c>
       <c r="O7">
-        <v>4.5400000000000003E-2</v>
+        <v>0.0496</v>
       </c>
       <c r="P7">
         <v>1</v>
@@ -975,25 +880,25 @@
         <v>1</v>
       </c>
       <c r="R7">
-        <v>0.442</v>
+        <v>0.456</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>0.234</v>
       </c>
       <c r="T7">
-        <v>0</v>
+        <v>0.31</v>
       </c>
       <c r="U7">
-        <v>0.86799999999999999</v>
+        <v>0.916</v>
       </c>
       <c r="V7">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="W7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.052</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8">
         <v>1000</v>
       </c>
@@ -1004,40 +909,40 @@
         <v>0.6</v>
       </c>
       <c r="D8">
-        <v>2.0011000000000001</v>
+        <v>1.9968</v>
       </c>
       <c r="E8">
-        <v>1.1000000000000001E-3</v>
+        <v>-0.0032</v>
       </c>
       <c r="F8">
-        <v>2.8E-3</v>
+        <v>0.0031</v>
       </c>
       <c r="G8">
-        <v>0.49919999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="H8">
-        <v>-8.0000000000000004E-4</v>
+        <v>-0</v>
       </c>
       <c r="I8">
-        <v>6.9999999999999999E-4</v>
+        <v>0.0008</v>
       </c>
       <c r="J8">
-        <v>5.0603999999999996</v>
+        <v>5.0573</v>
       </c>
       <c r="K8">
-        <v>6.0400000000000002E-2</v>
+        <v>0.0573</v>
       </c>
       <c r="L8">
-        <v>0.2198</v>
+        <v>0.2397</v>
       </c>
       <c r="M8">
-        <v>0.60140000000000005</v>
+        <v>0.5985</v>
       </c>
       <c r="N8">
-        <v>1.4E-3</v>
+        <v>-0.0015</v>
       </c>
       <c r="O8">
-        <v>1.6000000000000001E-3</v>
+        <v>0.0014</v>
       </c>
       <c r="P8">
         <v>1</v>
@@ -1049,22 +954,22 @@
         <v>0</v>
       </c>
       <c r="S8">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="T8">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="U8">
         <v>0</v>
       </c>
       <c r="V8">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="W8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -1075,40 +980,40 @@
         <v>0.9</v>
       </c>
       <c r="D9">
-        <v>2.0013000000000001</v>
+        <v>1.9997</v>
       </c>
       <c r="E9">
-        <v>1.2999999999999999E-3</v>
+        <v>-0.0003</v>
       </c>
       <c r="F9">
-        <v>1.8E-3</v>
+        <v>0.0017</v>
       </c>
       <c r="G9">
-        <v>0.49809999999999999</v>
+        <v>0.2475</v>
       </c>
       <c r="H9">
-        <v>-1.9E-3</v>
+        <v>-0.0025</v>
       </c>
       <c r="I9">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0003</v>
       </c>
       <c r="J9">
-        <v>5.0483000000000002</v>
+        <v>5.0357</v>
       </c>
       <c r="K9">
-        <v>4.8300000000000003E-2</v>
+        <v>0.0357</v>
       </c>
       <c r="L9">
-        <v>0.31090000000000001</v>
+        <v>0.3125</v>
       </c>
       <c r="M9">
-        <v>0.89600000000000002</v>
+        <v>0.8951</v>
       </c>
       <c r="N9">
-        <v>-4.0000000000000001E-3</v>
+        <v>-0.0049</v>
       </c>
       <c r="O9">
-        <v>5.9999999999999995E-4</v>
+        <v>0.0005</v>
       </c>
       <c r="P9">
         <v>1</v>
@@ -1120,22 +1025,22 @@
         <v>0</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>0.512</v>
       </c>
       <c r="T9">
-        <v>0</v>
+        <v>0.488</v>
       </c>
       <c r="U9">
         <v>0</v>
       </c>
       <c r="V9">
-        <v>0</v>
+        <v>0.512</v>
       </c>
       <c r="W9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.488</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10">
         <v>10000</v>
       </c>
@@ -1146,40 +1051,40 @@
         <v>0.6</v>
       </c>
       <c r="D10">
-        <v>1.9994000000000001</v>
+        <v>2.0009</v>
       </c>
       <c r="E10">
-        <v>-5.9999999999999995E-4</v>
+        <v>0.0009</v>
       </c>
       <c r="F10">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0002</v>
       </c>
       <c r="G10">
-        <v>0.4995</v>
+        <v>0.249</v>
       </c>
       <c r="H10">
-        <v>-5.0000000000000001E-4</v>
+        <v>-0.001</v>
       </c>
       <c r="I10">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0003</v>
       </c>
       <c r="J10">
-        <v>2.0270000000000001</v>
+        <v>2.0273</v>
       </c>
       <c r="K10">
-        <v>2.7E-2</v>
+        <v>0.0273</v>
       </c>
       <c r="L10">
-        <v>8.5000000000000006E-3</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="M10">
-        <v>0.60329999999999995</v>
+        <v>0.6006</v>
       </c>
       <c r="N10">
-        <v>3.3E-3</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="O10">
-        <v>6.8999999999999999E-3</v>
+        <v>0.0063</v>
       </c>
       <c r="P10">
         <v>1</v>
@@ -1191,22 +1096,22 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>0</v>
+        <v>0.512</v>
       </c>
       <c r="T10">
-        <v>0</v>
+        <v>0.488</v>
       </c>
       <c r="U10">
         <v>0</v>
       </c>
       <c r="V10">
-        <v>0</v>
+        <v>0.512</v>
       </c>
       <c r="W10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.488</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11">
         <v>10000</v>
       </c>
@@ -1217,40 +1122,40 @@
         <v>0.9</v>
       </c>
       <c r="D11">
-        <v>2.0003000000000002</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>2.9999999999999997E-4</v>
+        <v>-0</v>
       </c>
       <c r="F11">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0002</v>
       </c>
       <c r="G11">
-        <v>0.49719999999999998</v>
+        <v>0.2468</v>
       </c>
       <c r="H11">
-        <v>-2.8E-3</v>
+        <v>-0.0032</v>
       </c>
       <c r="I11">
-        <v>1E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="J11">
-        <v>2.0356999999999998</v>
+        <v>2.013</v>
       </c>
       <c r="K11">
-        <v>3.5700000000000003E-2</v>
+        <v>0.013</v>
       </c>
       <c r="L11">
-        <v>5.8599999999999999E-2</v>
+        <v>0.058</v>
       </c>
       <c r="M11">
-        <v>0.87529999999999997</v>
+        <v>0.8704</v>
       </c>
       <c r="N11">
-        <v>-2.47E-2</v>
+        <v>-0.0296</v>
       </c>
       <c r="O11">
-        <v>7.1000000000000004E-3</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="P11">
         <v>1</v>
@@ -1262,22 +1167,22 @@
         <v>0</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>0.438</v>
       </c>
       <c r="T11">
-        <v>0</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="U11">
-        <v>0.02</v>
+        <v>0.026</v>
       </c>
       <c r="V11">
-        <v>0</v>
+        <v>0.426</v>
       </c>
       <c r="W11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.548</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12">
         <v>10000</v>
       </c>
@@ -1288,40 +1193,40 @@
         <v>0.6</v>
       </c>
       <c r="D12">
-        <v>2.0001000000000002</v>
+        <v>1.9996</v>
       </c>
       <c r="E12">
-        <v>1E-4</v>
+        <v>-0.0004</v>
       </c>
       <c r="F12">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0003</v>
       </c>
       <c r="G12">
-        <v>0.50049999999999994</v>
+        <v>0.2501</v>
       </c>
       <c r="H12">
-        <v>5.0000000000000001E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="I12">
-        <v>1E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="J12">
-        <v>5.0007000000000001</v>
+        <v>5.0027</v>
       </c>
       <c r="K12">
-        <v>6.9999999999999999E-4</v>
+        <v>0.0027</v>
       </c>
       <c r="L12">
-        <v>2.2200000000000001E-2</v>
+        <v>0.0212</v>
       </c>
       <c r="M12">
-        <v>0.60070000000000001</v>
+        <v>0.5999</v>
       </c>
       <c r="N12">
-        <v>6.9999999999999999E-4</v>
+        <v>-0.0001</v>
       </c>
       <c r="O12">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="P12">
         <v>1</v>
@@ -1333,22 +1238,22 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>0</v>
+        <v>0.494</v>
       </c>
       <c r="T12">
-        <v>0</v>
+        <v>0.506</v>
       </c>
       <c r="U12">
         <v>0</v>
       </c>
       <c r="V12">
-        <v>0</v>
+        <v>0.494</v>
       </c>
       <c r="W12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.506</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13">
         <v>10000</v>
       </c>
@@ -1359,40 +1264,40 @@
         <v>0.9</v>
       </c>
       <c r="D13">
-        <v>2.0005000000000002</v>
+        <v>2.0004</v>
       </c>
       <c r="E13">
-        <v>5.0000000000000001E-4</v>
+        <v>0.0004</v>
       </c>
       <c r="F13">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0002</v>
       </c>
       <c r="G13">
-        <v>0.49990000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="H13">
-        <v>-1E-4</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <v>4.9970999999999997</v>
+        <v>5.001</v>
       </c>
       <c r="K13">
-        <v>-2.8999999999999998E-3</v>
+        <v>0.001</v>
       </c>
       <c r="L13">
-        <v>3.2500000000000001E-2</v>
+        <v>0.0292</v>
       </c>
       <c r="M13">
-        <v>0.89929999999999999</v>
+        <v>0.8996</v>
       </c>
       <c r="N13">
-        <v>-6.9999999999999999E-4</v>
+        <v>-0.0004</v>
       </c>
       <c r="O13">
-        <v>1E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="P13">
         <v>1</v>
@@ -1404,19 +1309,19 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>0.528</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>0.472</v>
       </c>
       <c r="U13">
         <v>0</v>
       </c>
       <c r="V13">
-        <v>0</v>
+        <v>0.528</v>
       </c>
       <c r="W13">
-        <v>0</v>
+        <v>0.472</v>
       </c>
     </row>
   </sheetData>
@@ -1425,61 +1330,73 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_true</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>epsilon_true</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_valid_gap</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mean_logLik_gap</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>min_logLik_gap</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>max_logLik_gap</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>mean_abs_logLik_gap</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>prop_gap_gt_small</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>prop_gap_gt_large</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>n_reg_better_reps</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>n_mode_better_reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2">
         <v>100</v>
       </c>
@@ -1493,31 +1410,31 @@
         <v>500</v>
       </c>
       <c r="E2">
-        <v>-2.0000000000000002E-5</v>
+        <v>3E-05</v>
       </c>
       <c r="F2">
-        <v>-5.5199999999999997E-3</v>
+        <v>-0.00731</v>
       </c>
       <c r="G2">
-        <v>2.8400000000000001E-3</v>
+        <v>0.01317</v>
       </c>
       <c r="H2">
-        <v>4.0000000000000003E-5</v>
+        <v>6.999999999999999E-05</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="L2">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3">
         <v>100</v>
       </c>
@@ -1531,16 +1448,16 @@
         <v>500</v>
       </c>
       <c r="E3">
-        <v>1.0000000000000001E-5</v>
+        <v>-0</v>
       </c>
       <c r="F3">
-        <v>-9.8999999999999999E-4</v>
+        <v>-0.00107</v>
       </c>
       <c r="G3">
-        <v>3.9399999999999999E-3</v>
+        <v>0.00136</v>
       </c>
       <c r="H3">
-        <v>2.0000000000000002E-5</v>
+        <v>1E-05</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1549,13 +1466,13 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="L3">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4">
         <v>100</v>
       </c>
@@ -1569,10 +1486,10 @@
         <v>500</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1587,13 +1504,13 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="L4">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5">
         <v>100</v>
       </c>
@@ -1610,10 +1527,10 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1E-05</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1625,13 +1542,13 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="L5">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6">
         <v>1000</v>
       </c>
@@ -1645,31 +1562,31 @@
         <v>500</v>
       </c>
       <c r="E6">
-        <v>6.0000000000000002E-5</v>
+        <v>-1E-05</v>
       </c>
       <c r="F6">
-        <v>-9.7000000000000005E-4</v>
+        <v>-0.01062</v>
       </c>
       <c r="G6">
-        <v>2.316E-2</v>
+        <v>0.00527</v>
       </c>
       <c r="H6">
-        <v>8.0000000000000007E-5</v>
+        <v>6E-05</v>
       </c>
       <c r="I6">
-        <v>2E-3</v>
+        <v>0.002</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="L6">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -1683,31 +1600,31 @@
         <v>500</v>
       </c>
       <c r="E7">
-        <v>2.0000000000000002E-5</v>
+        <v>-0.00031</v>
       </c>
       <c r="F7">
-        <v>-5.1999999999999995E-4</v>
+        <v>-0.16184</v>
       </c>
       <c r="G7">
-        <v>2.14E-3</v>
+        <v>0.01223</v>
       </c>
       <c r="H7">
-        <v>3.0000000000000001E-5</v>
+        <v>0.00041</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="L7">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8">
         <v>1000</v>
       </c>
@@ -1724,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-2.0000000000000002E-5</v>
+        <v>-2E-05</v>
       </c>
       <c r="G8">
-        <v>5.0000000000000002E-5</v>
+        <v>1E-05</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1739,13 +1656,13 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="L8">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -1759,13 +1676,13 @@
         <v>500</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F9">
-        <v>-1.0000000000000001E-5</v>
+        <v>-1E-05</v>
       </c>
       <c r="G9">
-        <v>1.0000000000000001E-5</v>
+        <v>1E-05</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1783,7 +1700,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10">
         <v>10000</v>
       </c>
@@ -1797,16 +1714,16 @@
         <v>500</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>-1E-05</v>
       </c>
       <c r="F10">
-        <v>-2.8800000000000002E-3</v>
+        <v>-0.00306</v>
       </c>
       <c r="G10">
-        <v>3.8E-3</v>
+        <v>0.00313</v>
       </c>
       <c r="H10">
-        <v>1E-4</v>
+        <v>0.00012</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1815,13 +1732,13 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="L10">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11">
         <v>10000</v>
       </c>
@@ -1835,16 +1752,16 @@
         <v>500</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>-1E-05</v>
       </c>
       <c r="F11">
-        <v>-2.4000000000000001E-4</v>
+        <v>-0.00239</v>
       </c>
       <c r="G11">
-        <v>1.06E-3</v>
+        <v>0.00039</v>
       </c>
       <c r="H11">
-        <v>4.0000000000000003E-5</v>
+        <v>4E-05</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -1853,13 +1770,13 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="L11">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12">
         <v>10000</v>
       </c>
@@ -1876,13 +1793,13 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>-1.7000000000000001E-4</v>
+        <v>-0.00014</v>
       </c>
       <c r="G12">
-        <v>1.4999999999999999E-4</v>
+        <v>0.00012</v>
       </c>
       <c r="H12">
-        <v>4.0000000000000003E-5</v>
+        <v>3E-05</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -1891,13 +1808,13 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L12">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13">
         <v>10000</v>
       </c>
@@ -1914,13 +1831,13 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>-1.2E-4</v>
+        <v>-8.000000000000001E-05</v>
       </c>
       <c r="G13">
-        <v>1E-4</v>
+        <v>0.00012</v>
       </c>
       <c r="H13">
-        <v>3.0000000000000001E-5</v>
+        <v>3E-05</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1929,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="L13">
-        <v>252</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>